<commit_message>
Switch September comparison to weekly-report (week-ending Thursday) basis
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014C1eqUA7BFiHff24GT8PwE
</commit_message>
<xml_diff>
--- a/Soybean_Inspections_Sep_Oct_2025_vs_2026.xlsx
+++ b/Soybean_Inspections_Sep_Oct_2025_vs_2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="September (Cert Date 1–30 Sep)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="September" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 October" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -116,9 +116,9 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -505,7 +505,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>US Soybean Export Inspections — Sept 2025 vs Sept 2026</t>
+          <t>US Soybean Export Inspections — September, weekly-report basis: weeks ending Thu 4/11/18/25 Sep 2025 vs Thu 3/10/17/24 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -586,10 +586,10 @@
         <v>0</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>2210969</v>
+        <v>1581810</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>2210969</v>
+        <v>1581810</v>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
@@ -600,38 +600,38 @@
         <v>0</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>34</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>ALGERIA</t>
+          <t>EGYPT</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>88670</v>
+        <v>392308</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>219250</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>130580</v>
-      </c>
-      <c r="E7" s="8" t="n">
-        <v>1.473</v>
+        <v>287000</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>-105308</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>-0.268</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="H7" s="6" t="n">
-        <v>3</v>
+      <c r="H7" s="8" t="n">
+        <v>-2</v>
       </c>
     </row>
     <row r="8">
@@ -641,137 +641,137 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>427278</v>
+        <v>332913</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>209008</v>
-      </c>
-      <c r="D8" s="9" t="n">
-        <v>-218270</v>
-      </c>
-      <c r="E8" s="10" t="n">
-        <v>-0.511</v>
+        <v>196733</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>-136180</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>-0.409</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>37</v>
-      </c>
-      <c r="H8" s="9" t="n">
-        <v>-1</v>
+        <v>36</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>-3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>EGYPT</t>
+          <t>JAPAN</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>516125</v>
+        <v>257479</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>171813</v>
-      </c>
-      <c r="D9" s="9" t="n">
-        <v>-344312</v>
-      </c>
-      <c r="E9" s="10" t="n">
-        <v>-0.667</v>
+        <v>170766</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>-86713</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>-0.337</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H9" s="9" t="n">
-        <v>-6</v>
+        <v>31</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>JAPAN</t>
+          <t>ITALY</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>237249</v>
+        <v>185744</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>167485</v>
-      </c>
-      <c r="D10" s="9" t="n">
-        <v>-69764</v>
-      </c>
-      <c r="E10" s="10" t="n">
-        <v>-0.294</v>
+        <v>162784</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>-22960</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>-0.124</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>28</v>
-      </c>
-      <c r="H10" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>ITALY</t>
+          <t>INDONESIA</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>185744</v>
+        <v>188108</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>162784</v>
-      </c>
-      <c r="D11" s="9" t="n">
-        <v>-22960</v>
-      </c>
-      <c r="E11" s="10" t="n">
-        <v>-0.124</v>
+        <v>133674</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>-54434</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>-0.289</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>3</v>
+        <v>212</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>0</v>
+        <v>231</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>INDONESIA</t>
+          <t>ALGERIA</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>210410</v>
+        <v>88670</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>131617</v>
-      </c>
-      <c r="D12" s="9" t="n">
-        <v>-78793</v>
+        <v>128695</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>40025</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>-0.374</v>
+        <v>0.451</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>278</v>
+        <v>2</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>225</v>
-      </c>
-      <c r="H12" s="9" t="n">
-        <v>-53</v>
+        <v>3</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -786,10 +786,10 @@
       <c r="C13" s="5" t="n">
         <v>114598</v>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="8" t="n">
         <v>-54933</v>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="9" t="n">
         <v>-0.324</v>
       </c>
       <c r="F13" s="5" t="n">
@@ -798,7 +798,7 @@
       <c r="G13" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H13" s="9" t="n">
+      <c r="H13" s="8" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -814,10 +814,10 @@
       <c r="C14" s="5" t="n">
         <v>59652</v>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="8" t="n">
         <v>-9436</v>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E14" s="9" t="n">
         <v>-0.137</v>
       </c>
       <c r="F14" s="5" t="n">
@@ -840,13 +840,13 @@
         <v>128961</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>58993</v>
-      </c>
-      <c r="D15" s="9" t="n">
-        <v>-69968</v>
-      </c>
-      <c r="E15" s="10" t="n">
-        <v>-0.5429999999999999</v>
+        <v>58374</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>-70587</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>-0.547</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>2</v>
@@ -854,7 +854,7 @@
       <c r="G15" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="9" t="n">
+      <c r="H15" s="8" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -865,25 +865,25 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>34392</v>
+        <v>30794</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>40636</v>
+        <v>40096</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>6244</v>
-      </c>
-      <c r="E16" s="8" t="n">
-        <v>0.182</v>
+        <v>9302</v>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>0.302</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17">
@@ -893,16 +893,16 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>30425</v>
+        <v>27740</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>36416</v>
+        <v>33430</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>5991</v>
-      </c>
-      <c r="E17" s="8" t="n">
-        <v>0.197</v>
+        <v>5690</v>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>0.205</v>
       </c>
       <c r="F17" s="5" t="n">
         <v>3</v>
@@ -917,201 +917,201 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>PORTUGAL</t>
+          <t>TAIWAN</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>0</v>
+        <v>85344</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>35887</v>
-      </c>
-      <c r="D18" s="6" t="n">
-        <v>35887</v>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
+        <v>32370</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>-52974</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>-0.621</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0</v>
+        <v>233</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H18" s="6" t="n">
-        <v>1</v>
+        <v>96</v>
+      </c>
+      <c r="H18" s="8" t="n">
+        <v>-137</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>TAIWAN</t>
+          <t>MALAYSIA</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>99132</v>
+        <v>43375</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>31293</v>
-      </c>
-      <c r="D19" s="9" t="n">
-        <v>-67839</v>
-      </c>
-      <c r="E19" s="10" t="n">
-        <v>-0.6840000000000001</v>
+        <v>22653</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>-20722</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>-0.478</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>269</v>
+        <v>117</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>90</v>
-      </c>
-      <c r="H19" s="9" t="n">
-        <v>-179</v>
+        <v>60</v>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>-57</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>MALAYSIA</t>
+          <t>COSTA RICA</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>45137</v>
+        <v>25355</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>21184</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>-23953</v>
-      </c>
-      <c r="E20" s="10" t="n">
-        <v>-0.531</v>
+        <v>12500</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>-12855</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>-0.507</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>121</v>
+        <v>2</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>57</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>-64</v>
+        <v>1</v>
+      </c>
+      <c r="H20" s="8" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>COSTA RICA</t>
+          <t>SAUDI ARABIA</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>24505</v>
+        <v>0</v>
       </c>
       <c r="C21" s="5" t="n">
-        <v>19696</v>
-      </c>
-      <c r="D21" s="9" t="n">
-        <v>-4809</v>
-      </c>
-      <c r="E21" s="10" t="n">
-        <v>-0.196</v>
+        <v>9853</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>9853</v>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
       </c>
       <c r="F21" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H21" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>SAUDI ARABIA</t>
+          <t>CANADA</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>0</v>
+        <v>1996</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>9853</v>
+        <v>7963</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>9853</v>
-      </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
+        <v>5967</v>
+      </c>
+      <c r="E22" s="10" t="n">
+        <v>2.989</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G22" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="6" t="n">
-        <v>1</v>
+      <c r="H22" s="8" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>CANADA</t>
+          <t>PHILIPPINES</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>1996</v>
+        <v>11038</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>7963</v>
-      </c>
-      <c r="D23" s="6" t="n">
-        <v>5967</v>
-      </c>
-      <c r="E23" s="8" t="n">
-        <v>2.989</v>
+        <v>6656</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>-4382</v>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>-0.397</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H23" s="9" t="n">
-        <v>-1</v>
+        <v>26</v>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>-14</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>PHILIPPINES</t>
+          <t>PANAMA</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>10402</v>
+        <v>0</v>
       </c>
       <c r="C24" s="5" t="n">
-        <v>6729</v>
-      </c>
-      <c r="D24" s="9" t="n">
-        <v>-3673</v>
-      </c>
-      <c r="E24" s="10" t="n">
-        <v>-0.353</v>
+        <v>4001</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>4001</v>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
       </c>
       <c r="F24" s="5" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>26</v>
-      </c>
-      <c r="H24" s="9" t="n">
-        <v>-10</v>
+        <v>1</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -1121,215 +1121,213 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>20054</v>
+        <v>17262</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>4579</v>
-      </c>
-      <c r="D25" s="9" t="n">
-        <v>-15475</v>
-      </c>
-      <c r="E25" s="10" t="n">
-        <v>-0.772</v>
+        <v>3992</v>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>-13270</v>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>-0.769</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="G25" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="H25" s="9" t="n">
-        <v>-55</v>
+        <v>11</v>
+      </c>
+      <c r="H25" s="8" t="n">
+        <v>-49</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>PANAMA</t>
+          <t>KOREA REP</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>0</v>
+        <v>342</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>4001</v>
+        <v>1685</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>4001</v>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
+        <v>1343</v>
+      </c>
+      <c r="E26" s="10" t="n">
+        <v>3.927</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>KOREA REP</t>
+          <t>CAMBODIA</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>880</v>
+        <v>2347</v>
       </c>
       <c r="C27" s="5" t="n">
-        <v>1906</v>
-      </c>
-      <c r="D27" s="6" t="n">
-        <v>1026</v>
-      </c>
-      <c r="E27" s="8" t="n">
-        <v>1.166</v>
+        <v>1225</v>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>-1122</v>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>-0.478</v>
       </c>
       <c r="F27" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="G27" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="G27" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="H27" s="6" t="n">
-        <v>7</v>
+      <c r="H27" s="8" t="n">
+        <v>-8</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>CAMBODIA</t>
+          <t>SINGAPORE</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>2543</v>
+        <v>0</v>
       </c>
       <c r="C28" s="5" t="n">
-        <v>1470</v>
-      </c>
-      <c r="D28" s="9" t="n">
-        <v>-1073</v>
-      </c>
-      <c r="E28" s="10" t="n">
-        <v>-0.422</v>
+        <v>245</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>245</v>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
       </c>
       <c r="F28" s="5" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="H28" s="9" t="n">
-        <v>-8</v>
+        <v>1</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>SINGAPORE</t>
+          <t>TURKEY</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>0</v>
+        <v>140323</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>245</v>
-      </c>
-      <c r="D29" s="6" t="n">
-        <v>245</v>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>-140323</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>-1</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G29" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H29" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="H29" s="8" t="n">
+        <v>-2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>TURKEY</t>
+          <t>SPAIN</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>209620</v>
+        <v>50899</v>
       </c>
       <c r="C30" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D30" s="9" t="n">
-        <v>-209620</v>
-      </c>
-      <c r="E30" s="10" t="n">
+      <c r="D30" s="8" t="n">
+        <v>-50899</v>
+      </c>
+      <c r="E30" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G30" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H30" s="9" t="n">
-        <v>-3</v>
+      <c r="H30" s="8" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>PAKISTAN</t>
+          <t>IRAQ</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>173686</v>
+        <v>52418</v>
       </c>
       <c r="C31" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D31" s="9" t="n">
-        <v>-173686</v>
-      </c>
-      <c r="E31" s="10" t="n">
+      <c r="D31" s="8" t="n">
+        <v>-52418</v>
+      </c>
+      <c r="E31" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G31" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="9" t="n">
-        <v>-3</v>
+      <c r="H31" s="8" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>SPAIN</t>
+          <t>PAKISTAN</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>50899</v>
+        <v>58648</v>
       </c>
       <c r="C32" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D32" s="9" t="n">
-        <v>-50899</v>
-      </c>
-      <c r="E32" s="10" t="n">
+      <c r="D32" s="8" t="n">
+        <v>-58648</v>
+      </c>
+      <c r="E32" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="F32" s="5" t="n">
@@ -1338,26 +1336,26 @@
       <c r="G32" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="9" t="n">
+      <c r="H32" s="8" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>IRAQ</t>
+          <t>UN KINGDOM</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>52418</v>
+        <v>67129</v>
       </c>
       <c r="C33" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D33" s="9" t="n">
-        <v>-52418</v>
-      </c>
-      <c r="E33" s="10" t="n">
+      <c r="D33" s="8" t="n">
+        <v>-67129</v>
+      </c>
+      <c r="E33" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="F33" s="5" t="n">
@@ -1366,26 +1364,26 @@
       <c r="G33" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="9" t="n">
+      <c r="H33" s="8" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>UN KINGDOM</t>
+          <t>VENEZUELA</t>
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>67129</v>
+        <v>7205</v>
       </c>
       <c r="C34" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D34" s="9" t="n">
-        <v>-67129</v>
-      </c>
-      <c r="E34" s="10" t="n">
+      <c r="D34" s="8" t="n">
+        <v>-7205</v>
+      </c>
+      <c r="E34" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="F34" s="5" t="n">
@@ -1394,7 +1392,7 @@
       <c r="G34" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="9" t="n">
+      <c r="H34" s="8" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -1410,10 +1408,10 @@
       <c r="C35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D35" s="9" t="n">
+      <c r="D35" s="8" t="n">
         <v>-29189</v>
       </c>
-      <c r="E35" s="10" t="n">
+      <c r="E35" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="F35" s="5" t="n">
@@ -1422,148 +1420,92 @@
       <c r="G35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="9" t="n">
+      <c r="H35" s="8" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>NEPAL</t>
+          <t>GRENADA</t>
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>1053</v>
+        <v>1000</v>
       </c>
       <c r="C36" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D36" s="9" t="n">
-        <v>-1053</v>
-      </c>
-      <c r="E36" s="10" t="n">
+      <c r="D36" s="8" t="n">
+        <v>-1000</v>
+      </c>
+      <c r="E36" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G36" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="9" t="n">
-        <v>-3</v>
+      <c r="H36" s="8" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>VENEZUELA</t>
+          <t>NEPAL</t>
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>7205</v>
+        <v>1347</v>
       </c>
       <c r="C37" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D37" s="9" t="n">
-        <v>-7205</v>
-      </c>
-      <c r="E37" s="10" t="n">
+      <c r="D37" s="8" t="n">
+        <v>-1347</v>
+      </c>
+      <c r="E37" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G37" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H37" s="9" t="n">
-        <v>-1</v>
+      <c r="H37" s="8" t="n">
+        <v>-4</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>SRI LANKA</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="n">
-        <v>294</v>
-      </c>
-      <c r="C38" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="9" t="n">
-        <v>-294</v>
-      </c>
-      <c r="E38" s="10" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F38" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G38" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" s="9" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>GRENADA</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C39" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" s="9" t="n">
-        <v>-1000</v>
-      </c>
-      <c r="E39" s="10" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F39" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G39" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" s="9" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="11" t="inlineStr">
+      <c r="A38" s="11" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B40" s="12" t="n">
-        <v>2895015</v>
-      </c>
-      <c r="C40" s="12" t="n">
-        <v>3728027</v>
-      </c>
-      <c r="D40" s="13" t="n">
-        <v>833012</v>
-      </c>
-      <c r="E40" s="14" t="n">
-        <v>0.288</v>
-      </c>
-      <c r="F40" s="12" t="n">
-        <v>1023</v>
-      </c>
-      <c r="G40" s="12" t="n">
-        <v>715</v>
-      </c>
-      <c r="H40" s="15" t="n">
-        <v>-308</v>
+      <c r="B38" s="12" t="n">
+        <v>2466553</v>
+      </c>
+      <c r="C38" s="12" t="n">
+        <v>3070755</v>
+      </c>
+      <c r="D38" s="13" t="n">
+        <v>604202</v>
+      </c>
+      <c r="E38" s="14" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="F38" s="12" t="n">
+        <v>892</v>
+      </c>
+      <c r="G38" s="12" t="n">
+        <v>718</v>
+      </c>
+      <c r="H38" s="15" t="n">
+        <v>-174</v>
       </c>
     </row>
   </sheetData>
@@ -1831,10 +1773,10 @@
       <c r="C11" s="5" t="n">
         <v>32033</v>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="8" t="n">
         <v>-185562</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="9" t="n">
         <v>-0.853</v>
       </c>
       <c r="F11" s="5" t="n">
@@ -1843,7 +1785,7 @@
       <c r="G11" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="H11" s="9" t="n">
+      <c r="H11" s="8" t="n">
         <v>-9</v>
       </c>
     </row>
@@ -1862,7 +1804,7 @@
       <c r="D12" s="6" t="n">
         <v>11433</v>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="10" t="n">
         <v>1.096</v>
       </c>
       <c r="F12" s="5" t="n">
@@ -1871,7 +1813,7 @@
       <c r="G12" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="H12" s="9" t="n">
+      <c r="H12" s="8" t="n">
         <v>-3</v>
       </c>
     </row>
@@ -1887,10 +1829,10 @@
       <c r="C13" s="5" t="n">
         <v>11065</v>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="8" t="n">
         <v>-1129</v>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="9" t="n">
         <v>-0.09300000000000001</v>
       </c>
       <c r="F13" s="5" t="n">
@@ -1918,7 +1860,7 @@
       <c r="D14" s="6" t="n">
         <v>4343</v>
       </c>
-      <c r="E14" s="8" t="n">
+      <c r="E14" s="10" t="n">
         <v>0.6909999999999999</v>
       </c>
       <c r="F14" s="5" t="n">
@@ -1943,10 +1885,10 @@
       <c r="C15" s="5" t="n">
         <v>7590</v>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="D15" s="8" t="n">
         <v>-36581</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E15" s="9" t="n">
         <v>-0.828</v>
       </c>
       <c r="F15" s="5" t="n">
@@ -1955,7 +1897,7 @@
       <c r="G15" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="H15" s="9" t="n">
+      <c r="H15" s="8" t="n">
         <v>-106</v>
       </c>
     </row>
@@ -1971,10 +1913,10 @@
       <c r="C16" s="5" t="n">
         <v>7196</v>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="8" t="n">
         <v>-5089</v>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E16" s="9" t="n">
         <v>-0.414</v>
       </c>
       <c r="F16" s="5" t="n">
@@ -1999,10 +1941,10 @@
       <c r="C17" s="5" t="n">
         <v>5777</v>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="D17" s="8" t="n">
         <v>-23123</v>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E17" s="9" t="n">
         <v>-0.8</v>
       </c>
       <c r="F17" s="5" t="n">
@@ -2011,7 +1953,7 @@
       <c r="G17" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="H17" s="9" t="n">
+      <c r="H17" s="8" t="n">
         <v>-58</v>
       </c>
     </row>
@@ -2027,10 +1969,10 @@
       <c r="C18" s="5" t="n">
         <v>2767</v>
       </c>
-      <c r="D18" s="9" t="n">
+      <c r="D18" s="8" t="n">
         <v>-3477</v>
       </c>
-      <c r="E18" s="10" t="n">
+      <c r="E18" s="9" t="n">
         <v>-0.5570000000000001</v>
       </c>
       <c r="F18" s="5" t="n">
@@ -2039,7 +1981,7 @@
       <c r="G18" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="H18" s="9" t="n">
+      <c r="H18" s="8" t="n">
         <v>-7</v>
       </c>
     </row>
@@ -2058,7 +2000,7 @@
       <c r="D19" s="6" t="n">
         <v>881</v>
       </c>
-      <c r="E19" s="8" t="n">
+      <c r="E19" s="10" t="n">
         <v>5.152</v>
       </c>
       <c r="F19" s="5" t="n">
@@ -2083,10 +2025,10 @@
       <c r="C20" s="5" t="n">
         <v>587</v>
       </c>
-      <c r="D20" s="9" t="n">
+      <c r="D20" s="8" t="n">
         <v>-4555</v>
       </c>
-      <c r="E20" s="10" t="n">
+      <c r="E20" s="9" t="n">
         <v>-0.8859999999999999</v>
       </c>
       <c r="F20" s="5" t="n">
@@ -2095,7 +2037,7 @@
       <c r="G20" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H20" s="9" t="n">
+      <c r="H20" s="8" t="n">
         <v>-14</v>
       </c>
     </row>
@@ -2111,10 +2053,10 @@
       <c r="C21" s="5" t="n">
         <v>343</v>
       </c>
-      <c r="D21" s="9" t="n">
+      <c r="D21" s="8" t="n">
         <v>-195</v>
       </c>
-      <c r="E21" s="10" t="n">
+      <c r="E21" s="9" t="n">
         <v>-0.362</v>
       </c>
       <c r="F21" s="5" t="n">
@@ -2123,7 +2065,7 @@
       <c r="G21" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="9" t="n">
+      <c r="H21" s="8" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -2139,10 +2081,10 @@
       <c r="C22" s="5" t="n">
         <v>245</v>
       </c>
-      <c r="D22" s="9" t="n">
+      <c r="D22" s="8" t="n">
         <v>-367</v>
       </c>
-      <c r="E22" s="10" t="n">
+      <c r="E22" s="9" t="n">
         <v>-0.6</v>
       </c>
       <c r="F22" s="5" t="n">
@@ -2151,26 +2093,26 @@
       <c r="G22" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="9" t="n">
+      <c r="H22" s="8" t="n">
         <v>-2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>ITALY</t>
+          <t>TURKEY</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>45900</v>
+        <v>69297</v>
       </c>
       <c r="C23" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D23" s="9" t="n">
-        <v>-45900</v>
-      </c>
-      <c r="E23" s="10" t="n">
+      <c r="D23" s="8" t="n">
+        <v>-69297</v>
+      </c>
+      <c r="E23" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="F23" s="5" t="n">
@@ -2179,64 +2121,64 @@
       <c r="G23" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="9" t="n">
+      <c r="H23" s="8" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>TURKEY</t>
+          <t>EGYPT</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>69297</v>
+        <v>181571</v>
       </c>
       <c r="C24" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D24" s="9" t="n">
-        <v>-69297</v>
-      </c>
-      <c r="E24" s="10" t="n">
+      <c r="D24" s="8" t="n">
+        <v>-181571</v>
+      </c>
+      <c r="E24" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G24" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="9" t="n">
-        <v>-1</v>
+      <c r="H24" s="8" t="n">
+        <v>-3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>EGYPT</t>
+          <t>ITALY</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>181571</v>
+        <v>45900</v>
       </c>
       <c r="C25" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D25" s="9" t="n">
-        <v>-181571</v>
-      </c>
-      <c r="E25" s="10" t="n">
+      <c r="D25" s="8" t="n">
+        <v>-45900</v>
+      </c>
+      <c r="E25" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G25" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="9" t="n">
-        <v>-3</v>
+      <c r="H25" s="8" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="26">
@@ -2251,10 +2193,10 @@
       <c r="C26" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D26" s="9" t="n">
+      <c r="D26" s="8" t="n">
         <v>-115038</v>
       </c>
-      <c r="E26" s="10" t="n">
+      <c r="E26" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="F26" s="5" t="n">
@@ -2263,26 +2205,26 @@
       <c r="G26" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H26" s="9" t="n">
+      <c r="H26" s="8" t="n">
         <v>-2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>SRI LANKA</t>
+          <t>DOMINICN REP</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>294</v>
+        <v>4958</v>
       </c>
       <c r="C27" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D27" s="9" t="n">
-        <v>-294</v>
-      </c>
-      <c r="E27" s="10" t="n">
+      <c r="D27" s="8" t="n">
+        <v>-4958</v>
+      </c>
+      <c r="E27" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="F27" s="5" t="n">
@@ -2291,26 +2233,26 @@
       <c r="G27" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H27" s="9" t="n">
+      <c r="H27" s="8" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>DOMINICN REP</t>
+          <t>SAUDI ARABIA</t>
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>4958</v>
+        <v>21871</v>
       </c>
       <c r="C28" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D28" s="9" t="n">
-        <v>-4958</v>
-      </c>
-      <c r="E28" s="10" t="n">
+      <c r="D28" s="8" t="n">
+        <v>-21871</v>
+      </c>
+      <c r="E28" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="F28" s="5" t="n">
@@ -2319,26 +2261,26 @@
       <c r="G28" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="9" t="n">
+      <c r="H28" s="8" t="n">
         <v>-1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>SAUDI ARABIA</t>
+          <t>SRI LANKA</t>
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>21871</v>
+        <v>294</v>
       </c>
       <c r="C29" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D29" s="9" t="n">
-        <v>-21871</v>
-      </c>
-      <c r="E29" s="10" t="n">
+      <c r="D29" s="8" t="n">
+        <v>-294</v>
+      </c>
+      <c r="E29" s="9" t="n">
         <v>-1</v>
       </c>
       <c r="F29" s="5" t="n">
@@ -2347,7 +2289,7 @@
       <c r="G29" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="9" t="n">
+      <c r="H29" s="8" t="n">
         <v>-1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add China vs Rest of World summary to soybean comparison
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014C1eqUA7BFiHff24GT8PwE
</commit_message>
<xml_diff>
--- a/Soybean_Inspections_Sep_Oct_2025_vs_2026.xlsx
+++ b/Soybean_Inspections_Sep_Oct_2025_vs_2026.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="September" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 October" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary China vs RoW" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="September" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 October" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,9 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0;-#,##0;-"/>
     <numFmt numFmtId="165" formatCode="+0.0%;-0.0%;0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -103,12 +105,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -116,14 +118,23 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -489,7 +500,438 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>US Soybean Export Inspections — China vs Rest of World (weekly-report basis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sept = weeks ending 4–25 Sep 2025 / 3–24 Sep 2026; Week 1 Oct = week ending 2 Oct 2025 / 1 Oct 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>MT 2025</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>MT 2026</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Δ MT</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Δ %</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t># Insp 2025</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t># Insp 2026</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Δ Insp</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Share of MT 2025</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Share of MT 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>1581810</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>1581810</v>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="J5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="8" t="n">
+        <v>0.5151208741824079</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr"/>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Rest of World excl. China</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>2466553</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>1488945</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>-977608</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>-0.3963458316119702</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>892</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>694</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>-198</v>
+      </c>
+      <c r="J6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="8" t="n">
+        <v>0.4848791258175921</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr"/>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>2466553</v>
+      </c>
+      <c r="D7" s="12" t="n">
+        <v>3070755</v>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>604202</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0.2449580446882755</v>
+      </c>
+      <c r="G7" s="12" t="n">
+        <v>892</v>
+      </c>
+      <c r="H7" s="12" t="n">
+        <v>718</v>
+      </c>
+      <c r="I7" s="15" t="n">
+        <v>-174</v>
+      </c>
+      <c r="J7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Week 1 October</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>756492</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>756492</v>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="J8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="8" t="n">
+        <v>0.6645127967280854</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Rest of World excl. China</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>783495</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>381924</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>-401571</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>-0.5125380506576303</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>313</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>114</v>
+      </c>
+      <c r="I9" s="9" t="n">
+        <v>-199</v>
+      </c>
+      <c r="J9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="8" t="n">
+        <v>0.3354872032719147</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr"/>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>783495</v>
+      </c>
+      <c r="D10" s="12" t="n">
+        <v>1138416</v>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>354921</v>
+      </c>
+      <c r="F10" s="14" t="n">
+        <v>0.4529971473972393</v>
+      </c>
+      <c r="G10" s="12" t="n">
+        <v>313</v>
+      </c>
+      <c r="H10" s="12" t="n">
+        <v>126</v>
+      </c>
+      <c r="I10" s="15" t="n">
+        <v>-187</v>
+      </c>
+      <c r="J10" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Sept + Week 1 Oct</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>2338302</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>2338302</v>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="J11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="8" t="n">
+        <v>0.5555255417278129</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr"/>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Rest of World excl. China</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>3250048</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>1870869</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>-1379179</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>-0.4243565018116656</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>1205</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>808</v>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>-397</v>
+      </c>
+      <c r="J12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>0.4444744582721871</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr"/>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>3250048</v>
+      </c>
+      <c r="D13" s="12" t="n">
+        <v>4209171</v>
+      </c>
+      <c r="E13" s="13" t="n">
+        <v>959123</v>
+      </c>
+      <c r="F13" s="14" t="n">
+        <v>0.2951104106770115</v>
+      </c>
+      <c r="G13" s="12" t="n">
+        <v>1205</v>
+      </c>
+      <c r="H13" s="12" t="n">
+        <v>844</v>
+      </c>
+      <c r="I13" s="15" t="n">
+        <v>-361</v>
+      </c>
+      <c r="J13" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -517,60 +959,60 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Destination</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>Metric tons</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="C4" s="17" t="n"/>
+      <c r="D4" s="17" t="n"/>
+      <c r="E4" s="17" t="n"/>
+      <c r="F4" s="17" t="inlineStr">
         <is>
           <t>Number of inspections</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
+      <c r="G4" s="17" t="n"/>
+      <c r="H4" s="17" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="A5" s="17" t="n"/>
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>Δ MT</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>Δ %</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="17" t="inlineStr">
         <is>
           <t>Δ</t>
         </is>
@@ -618,10 +1060,10 @@
       <c r="C7" s="5" t="n">
         <v>287000</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="9" t="n">
         <v>-105308</v>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="E7" s="10" t="n">
         <v>-0.268</v>
       </c>
       <c r="F7" s="5" t="n">
@@ -630,7 +1072,7 @@
       <c r="G7" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="H7" s="9" t="n">
         <v>-2</v>
       </c>
     </row>
@@ -646,10 +1088,10 @@
       <c r="C8" s="5" t="n">
         <v>196733</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="9" t="n">
         <v>-136180</v>
       </c>
-      <c r="E8" s="9" t="n">
+      <c r="E8" s="10" t="n">
         <v>-0.409</v>
       </c>
       <c r="F8" s="5" t="n">
@@ -658,7 +1100,7 @@
       <c r="G8" s="5" t="n">
         <v>36</v>
       </c>
-      <c r="H8" s="8" t="n">
+      <c r="H8" s="9" t="n">
         <v>-3</v>
       </c>
     </row>
@@ -674,10 +1116,10 @@
       <c r="C9" s="5" t="n">
         <v>170766</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="9" t="n">
         <v>-86713</v>
       </c>
-      <c r="E9" s="9" t="n">
+      <c r="E9" s="10" t="n">
         <v>-0.337</v>
       </c>
       <c r="F9" s="5" t="n">
@@ -702,10 +1144,10 @@
       <c r="C10" s="5" t="n">
         <v>162784</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="9" t="n">
         <v>-22960</v>
       </c>
-      <c r="E10" s="9" t="n">
+      <c r="E10" s="10" t="n">
         <v>-0.124</v>
       </c>
       <c r="F10" s="5" t="n">
@@ -730,10 +1172,10 @@
       <c r="C11" s="5" t="n">
         <v>133674</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="9" t="n">
         <v>-54434</v>
       </c>
-      <c r="E11" s="9" t="n">
+      <c r="E11" s="10" t="n">
         <v>-0.289</v>
       </c>
       <c r="F11" s="5" t="n">
@@ -761,7 +1203,7 @@
       <c r="D12" s="6" t="n">
         <v>40025</v>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E12" s="18" t="n">
         <v>0.451</v>
       </c>
       <c r="F12" s="5" t="n">
@@ -786,10 +1228,10 @@
       <c r="C13" s="5" t="n">
         <v>114598</v>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D13" s="9" t="n">
         <v>-54933</v>
       </c>
-      <c r="E13" s="9" t="n">
+      <c r="E13" s="10" t="n">
         <v>-0.324</v>
       </c>
       <c r="F13" s="5" t="n">
@@ -798,7 +1240,7 @@
       <c r="G13" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H13" s="8" t="n">
+      <c r="H13" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -814,10 +1256,10 @@
       <c r="C14" s="5" t="n">
         <v>59652</v>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="D14" s="9" t="n">
         <v>-9436</v>
       </c>
-      <c r="E14" s="9" t="n">
+      <c r="E14" s="10" t="n">
         <v>-0.137</v>
       </c>
       <c r="F14" s="5" t="n">
@@ -842,10 +1284,10 @@
       <c r="C15" s="5" t="n">
         <v>58374</v>
       </c>
-      <c r="D15" s="8" t="n">
+      <c r="D15" s="9" t="n">
         <v>-70587</v>
       </c>
-      <c r="E15" s="9" t="n">
+      <c r="E15" s="10" t="n">
         <v>-0.547</v>
       </c>
       <c r="F15" s="5" t="n">
@@ -854,7 +1296,7 @@
       <c r="G15" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="8" t="n">
+      <c r="H15" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -873,7 +1315,7 @@
       <c r="D16" s="6" t="n">
         <v>9302</v>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E16" s="18" t="n">
         <v>0.302</v>
       </c>
       <c r="F16" s="5" t="n">
@@ -901,7 +1343,7 @@
       <c r="D17" s="6" t="n">
         <v>5690</v>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E17" s="18" t="n">
         <v>0.205</v>
       </c>
       <c r="F17" s="5" t="n">
@@ -926,10 +1368,10 @@
       <c r="C18" s="5" t="n">
         <v>32370</v>
       </c>
-      <c r="D18" s="8" t="n">
+      <c r="D18" s="9" t="n">
         <v>-52974</v>
       </c>
-      <c r="E18" s="9" t="n">
+      <c r="E18" s="10" t="n">
         <v>-0.621</v>
       </c>
       <c r="F18" s="5" t="n">
@@ -938,7 +1380,7 @@
       <c r="G18" s="5" t="n">
         <v>96</v>
       </c>
-      <c r="H18" s="8" t="n">
+      <c r="H18" s="9" t="n">
         <v>-137</v>
       </c>
     </row>
@@ -954,10 +1396,10 @@
       <c r="C19" s="5" t="n">
         <v>22653</v>
       </c>
-      <c r="D19" s="8" t="n">
+      <c r="D19" s="9" t="n">
         <v>-20722</v>
       </c>
-      <c r="E19" s="9" t="n">
+      <c r="E19" s="10" t="n">
         <v>-0.478</v>
       </c>
       <c r="F19" s="5" t="n">
@@ -966,7 +1408,7 @@
       <c r="G19" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="H19" s="8" t="n">
+      <c r="H19" s="9" t="n">
         <v>-57</v>
       </c>
     </row>
@@ -982,10 +1424,10 @@
       <c r="C20" s="5" t="n">
         <v>12500</v>
       </c>
-      <c r="D20" s="8" t="n">
+      <c r="D20" s="9" t="n">
         <v>-12855</v>
       </c>
-      <c r="E20" s="9" t="n">
+      <c r="E20" s="10" t="n">
         <v>-0.507</v>
       </c>
       <c r="F20" s="5" t="n">
@@ -994,7 +1436,7 @@
       <c r="G20" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H20" s="8" t="n">
+      <c r="H20" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -1043,7 +1485,7 @@
       <c r="D22" s="6" t="n">
         <v>5967</v>
       </c>
-      <c r="E22" s="10" t="n">
+      <c r="E22" s="18" t="n">
         <v>2.989</v>
       </c>
       <c r="F22" s="5" t="n">
@@ -1052,7 +1494,7 @@
       <c r="G22" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="8" t="n">
+      <c r="H22" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -1068,10 +1510,10 @@
       <c r="C23" s="5" t="n">
         <v>6656</v>
       </c>
-      <c r="D23" s="8" t="n">
+      <c r="D23" s="9" t="n">
         <v>-4382</v>
       </c>
-      <c r="E23" s="9" t="n">
+      <c r="E23" s="10" t="n">
         <v>-0.397</v>
       </c>
       <c r="F23" s="5" t="n">
@@ -1080,7 +1522,7 @@
       <c r="G23" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="H23" s="8" t="n">
+      <c r="H23" s="9" t="n">
         <v>-14</v>
       </c>
     </row>
@@ -1126,10 +1568,10 @@
       <c r="C25" s="5" t="n">
         <v>3992</v>
       </c>
-      <c r="D25" s="8" t="n">
+      <c r="D25" s="9" t="n">
         <v>-13270</v>
       </c>
-      <c r="E25" s="9" t="n">
+      <c r="E25" s="10" t="n">
         <v>-0.769</v>
       </c>
       <c r="F25" s="5" t="n">
@@ -1138,7 +1580,7 @@
       <c r="G25" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="H25" s="8" t="n">
+      <c r="H25" s="9" t="n">
         <v>-49</v>
       </c>
     </row>
@@ -1157,7 +1599,7 @@
       <c r="D26" s="6" t="n">
         <v>1343</v>
       </c>
-      <c r="E26" s="10" t="n">
+      <c r="E26" s="18" t="n">
         <v>3.927</v>
       </c>
       <c r="F26" s="5" t="n">
@@ -1182,10 +1624,10 @@
       <c r="C27" s="5" t="n">
         <v>1225</v>
       </c>
-      <c r="D27" s="8" t="n">
+      <c r="D27" s="9" t="n">
         <v>-1122</v>
       </c>
-      <c r="E27" s="9" t="n">
+      <c r="E27" s="10" t="n">
         <v>-0.478</v>
       </c>
       <c r="F27" s="5" t="n">
@@ -1194,7 +1636,7 @@
       <c r="G27" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="H27" s="8" t="n">
+      <c r="H27" s="9" t="n">
         <v>-8</v>
       </c>
     </row>
@@ -1240,10 +1682,10 @@
       <c r="C29" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D29" s="8" t="n">
+      <c r="D29" s="9" t="n">
         <v>-140323</v>
       </c>
-      <c r="E29" s="9" t="n">
+      <c r="E29" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="F29" s="5" t="n">
@@ -1252,7 +1694,7 @@
       <c r="G29" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="8" t="n">
+      <c r="H29" s="9" t="n">
         <v>-2</v>
       </c>
     </row>
@@ -1268,10 +1710,10 @@
       <c r="C30" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D30" s="8" t="n">
+      <c r="D30" s="9" t="n">
         <v>-50899</v>
       </c>
-      <c r="E30" s="9" t="n">
+      <c r="E30" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="F30" s="5" t="n">
@@ -1280,7 +1722,7 @@
       <c r="G30" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H30" s="8" t="n">
+      <c r="H30" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -1296,10 +1738,10 @@
       <c r="C31" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D31" s="8" t="n">
+      <c r="D31" s="9" t="n">
         <v>-52418</v>
       </c>
-      <c r="E31" s="9" t="n">
+      <c r="E31" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="F31" s="5" t="n">
@@ -1308,7 +1750,7 @@
       <c r="G31" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="8" t="n">
+      <c r="H31" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -1324,10 +1766,10 @@
       <c r="C32" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D32" s="8" t="n">
+      <c r="D32" s="9" t="n">
         <v>-58648</v>
       </c>
-      <c r="E32" s="9" t="n">
+      <c r="E32" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="F32" s="5" t="n">
@@ -1336,7 +1778,7 @@
       <c r="G32" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H32" s="8" t="n">
+      <c r="H32" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -1352,10 +1794,10 @@
       <c r="C33" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D33" s="8" t="n">
+      <c r="D33" s="9" t="n">
         <v>-67129</v>
       </c>
-      <c r="E33" s="9" t="n">
+      <c r="E33" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="F33" s="5" t="n">
@@ -1364,7 +1806,7 @@
       <c r="G33" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="8" t="n">
+      <c r="H33" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -1380,10 +1822,10 @@
       <c r="C34" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D34" s="8" t="n">
+      <c r="D34" s="9" t="n">
         <v>-7205</v>
       </c>
-      <c r="E34" s="9" t="n">
+      <c r="E34" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="F34" s="5" t="n">
@@ -1392,7 +1834,7 @@
       <c r="G34" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="8" t="n">
+      <c r="H34" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -1408,10 +1850,10 @@
       <c r="C35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D35" s="8" t="n">
+      <c r="D35" s="9" t="n">
         <v>-29189</v>
       </c>
-      <c r="E35" s="9" t="n">
+      <c r="E35" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="F35" s="5" t="n">
@@ -1420,7 +1862,7 @@
       <c r="G35" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H35" s="8" t="n">
+      <c r="H35" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -1436,10 +1878,10 @@
       <c r="C36" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D36" s="8" t="n">
+      <c r="D36" s="9" t="n">
         <v>-1000</v>
       </c>
-      <c r="E36" s="9" t="n">
+      <c r="E36" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="F36" s="5" t="n">
@@ -1448,7 +1890,7 @@
       <c r="G36" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H36" s="8" t="n">
+      <c r="H36" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -1464,10 +1906,10 @@
       <c r="C37" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D37" s="8" t="n">
+      <c r="D37" s="9" t="n">
         <v>-1347</v>
       </c>
-      <c r="E37" s="9" t="n">
+      <c r="E37" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="F37" s="5" t="n">
@@ -1476,7 +1918,7 @@
       <c r="G37" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H37" s="8" t="n">
+      <c r="H37" s="9" t="n">
         <v>-4</v>
       </c>
     </row>
@@ -1506,6 +1948,64 @@
       </c>
       <c r="H38" s="15" t="n">
         <v>-174</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="12" t="n">
+        <v>1581810</v>
+      </c>
+      <c r="D39" s="13" t="n">
+        <v>1581810</v>
+      </c>
+      <c r="E39" s="19" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F39" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="H39" s="13" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>Rest of World excl. China</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="n">
+        <v>2466553</v>
+      </c>
+      <c r="C40" s="12" t="n">
+        <v>1488945</v>
+      </c>
+      <c r="D40" s="15" t="n">
+        <v>-977608</v>
+      </c>
+      <c r="E40" s="20" t="n">
+        <v>-0.396</v>
+      </c>
+      <c r="F40" s="12" t="n">
+        <v>892</v>
+      </c>
+      <c r="G40" s="12" t="n">
+        <v>694</v>
+      </c>
+      <c r="H40" s="15" t="n">
+        <v>-198</v>
       </c>
     </row>
   </sheetData>
@@ -1518,13 +2018,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1552,60 +2052,60 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Destination</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>Metric tons</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="C4" s="17" t="n"/>
+      <c r="D4" s="17" t="n"/>
+      <c r="E4" s="17" t="n"/>
+      <c r="F4" s="17" t="inlineStr">
         <is>
           <t>Number of inspections</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
+      <c r="G4" s="17" t="n"/>
+      <c r="H4" s="17" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="A5" s="17" t="n"/>
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>Δ MT</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>Δ %</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="17" t="inlineStr">
         <is>
           <t>Δ</t>
         </is>
@@ -1773,10 +2273,10 @@
       <c r="C11" s="5" t="n">
         <v>32033</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="9" t="n">
         <v>-185562</v>
       </c>
-      <c r="E11" s="9" t="n">
+      <c r="E11" s="10" t="n">
         <v>-0.853</v>
       </c>
       <c r="F11" s="5" t="n">
@@ -1785,7 +2285,7 @@
       <c r="G11" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H11" s="9" t="n">
         <v>-9</v>
       </c>
     </row>
@@ -1804,7 +2304,7 @@
       <c r="D12" s="6" t="n">
         <v>11433</v>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E12" s="18" t="n">
         <v>1.096</v>
       </c>
       <c r="F12" s="5" t="n">
@@ -1813,7 +2313,7 @@
       <c r="G12" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="H12" s="8" t="n">
+      <c r="H12" s="9" t="n">
         <v>-3</v>
       </c>
     </row>
@@ -1829,10 +2329,10 @@
       <c r="C13" s="5" t="n">
         <v>11065</v>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D13" s="9" t="n">
         <v>-1129</v>
       </c>
-      <c r="E13" s="9" t="n">
+      <c r="E13" s="10" t="n">
         <v>-0.09300000000000001</v>
       </c>
       <c r="F13" s="5" t="n">
@@ -1860,7 +2360,7 @@
       <c r="D14" s="6" t="n">
         <v>4343</v>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E14" s="18" t="n">
         <v>0.6909999999999999</v>
       </c>
       <c r="F14" s="5" t="n">
@@ -1885,10 +2385,10 @@
       <c r="C15" s="5" t="n">
         <v>7590</v>
       </c>
-      <c r="D15" s="8" t="n">
+      <c r="D15" s="9" t="n">
         <v>-36581</v>
       </c>
-      <c r="E15" s="9" t="n">
+      <c r="E15" s="10" t="n">
         <v>-0.828</v>
       </c>
       <c r="F15" s="5" t="n">
@@ -1897,7 +2397,7 @@
       <c r="G15" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="H15" s="8" t="n">
+      <c r="H15" s="9" t="n">
         <v>-106</v>
       </c>
     </row>
@@ -1913,10 +2413,10 @@
       <c r="C16" s="5" t="n">
         <v>7196</v>
       </c>
-      <c r="D16" s="8" t="n">
+      <c r="D16" s="9" t="n">
         <v>-5089</v>
       </c>
-      <c r="E16" s="9" t="n">
+      <c r="E16" s="10" t="n">
         <v>-0.414</v>
       </c>
       <c r="F16" s="5" t="n">
@@ -1941,10 +2441,10 @@
       <c r="C17" s="5" t="n">
         <v>5777</v>
       </c>
-      <c r="D17" s="8" t="n">
+      <c r="D17" s="9" t="n">
         <v>-23123</v>
       </c>
-      <c r="E17" s="9" t="n">
+      <c r="E17" s="10" t="n">
         <v>-0.8</v>
       </c>
       <c r="F17" s="5" t="n">
@@ -1953,7 +2453,7 @@
       <c r="G17" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="H17" s="8" t="n">
+      <c r="H17" s="9" t="n">
         <v>-58</v>
       </c>
     </row>
@@ -1969,10 +2469,10 @@
       <c r="C18" s="5" t="n">
         <v>2767</v>
       </c>
-      <c r="D18" s="8" t="n">
+      <c r="D18" s="9" t="n">
         <v>-3477</v>
       </c>
-      <c r="E18" s="9" t="n">
+      <c r="E18" s="10" t="n">
         <v>-0.5570000000000001</v>
       </c>
       <c r="F18" s="5" t="n">
@@ -1981,7 +2481,7 @@
       <c r="G18" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="H18" s="8" t="n">
+      <c r="H18" s="9" t="n">
         <v>-7</v>
       </c>
     </row>
@@ -2000,7 +2500,7 @@
       <c r="D19" s="6" t="n">
         <v>881</v>
       </c>
-      <c r="E19" s="10" t="n">
+      <c r="E19" s="18" t="n">
         <v>5.152</v>
       </c>
       <c r="F19" s="5" t="n">
@@ -2025,10 +2525,10 @@
       <c r="C20" s="5" t="n">
         <v>587</v>
       </c>
-      <c r="D20" s="8" t="n">
+      <c r="D20" s="9" t="n">
         <v>-4555</v>
       </c>
-      <c r="E20" s="9" t="n">
+      <c r="E20" s="10" t="n">
         <v>-0.8859999999999999</v>
       </c>
       <c r="F20" s="5" t="n">
@@ -2037,7 +2537,7 @@
       <c r="G20" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="H20" s="8" t="n">
+      <c r="H20" s="9" t="n">
         <v>-14</v>
       </c>
     </row>
@@ -2053,10 +2553,10 @@
       <c r="C21" s="5" t="n">
         <v>343</v>
       </c>
-      <c r="D21" s="8" t="n">
+      <c r="D21" s="9" t="n">
         <v>-195</v>
       </c>
-      <c r="E21" s="9" t="n">
+      <c r="E21" s="10" t="n">
         <v>-0.362</v>
       </c>
       <c r="F21" s="5" t="n">
@@ -2065,7 +2565,7 @@
       <c r="G21" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="8" t="n">
+      <c r="H21" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -2081,10 +2581,10 @@
       <c r="C22" s="5" t="n">
         <v>245</v>
       </c>
-      <c r="D22" s="8" t="n">
+      <c r="D22" s="9" t="n">
         <v>-367</v>
       </c>
-      <c r="E22" s="9" t="n">
+      <c r="E22" s="10" t="n">
         <v>-0.6</v>
       </c>
       <c r="F22" s="5" t="n">
@@ -2093,7 +2593,7 @@
       <c r="G22" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="8" t="n">
+      <c r="H22" s="9" t="n">
         <v>-2</v>
       </c>
     </row>
@@ -2109,10 +2609,10 @@
       <c r="C23" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D23" s="8" t="n">
+      <c r="D23" s="9" t="n">
         <v>-69297</v>
       </c>
-      <c r="E23" s="9" t="n">
+      <c r="E23" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="F23" s="5" t="n">
@@ -2121,7 +2621,7 @@
       <c r="G23" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="8" t="n">
+      <c r="H23" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -2137,10 +2637,10 @@
       <c r="C24" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D24" s="8" t="n">
+      <c r="D24" s="9" t="n">
         <v>-181571</v>
       </c>
-      <c r="E24" s="9" t="n">
+      <c r="E24" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="F24" s="5" t="n">
@@ -2149,7 +2649,7 @@
       <c r="G24" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="8" t="n">
+      <c r="H24" s="9" t="n">
         <v>-3</v>
       </c>
     </row>
@@ -2165,10 +2665,10 @@
       <c r="C25" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D25" s="8" t="n">
+      <c r="D25" s="9" t="n">
         <v>-45900</v>
       </c>
-      <c r="E25" s="9" t="n">
+      <c r="E25" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="F25" s="5" t="n">
@@ -2177,7 +2677,7 @@
       <c r="G25" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="8" t="n">
+      <c r="H25" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -2193,10 +2693,10 @@
       <c r="C26" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D26" s="8" t="n">
+      <c r="D26" s="9" t="n">
         <v>-115038</v>
       </c>
-      <c r="E26" s="9" t="n">
+      <c r="E26" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="F26" s="5" t="n">
@@ -2205,7 +2705,7 @@
       <c r="G26" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H26" s="8" t="n">
+      <c r="H26" s="9" t="n">
         <v>-2</v>
       </c>
     </row>
@@ -2221,10 +2721,10 @@
       <c r="C27" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D27" s="8" t="n">
+      <c r="D27" s="9" t="n">
         <v>-4958</v>
       </c>
-      <c r="E27" s="9" t="n">
+      <c r="E27" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="F27" s="5" t="n">
@@ -2233,7 +2733,7 @@
       <c r="G27" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H27" s="8" t="n">
+      <c r="H27" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -2249,10 +2749,10 @@
       <c r="C28" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D28" s="8" t="n">
+      <c r="D28" s="9" t="n">
         <v>-21871</v>
       </c>
-      <c r="E28" s="9" t="n">
+      <c r="E28" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="F28" s="5" t="n">
@@ -2261,7 +2761,7 @@
       <c r="G28" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H28" s="8" t="n">
+      <c r="H28" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -2277,10 +2777,10 @@
       <c r="C29" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D29" s="8" t="n">
+      <c r="D29" s="9" t="n">
         <v>-294</v>
       </c>
-      <c r="E29" s="9" t="n">
+      <c r="E29" s="10" t="n">
         <v>-1</v>
       </c>
       <c r="F29" s="5" t="n">
@@ -2289,7 +2789,7 @@
       <c r="G29" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H29" s="8" t="n">
+      <c r="H29" s="9" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -2319,6 +2819,64 @@
       </c>
       <c r="H30" s="15" t="n">
         <v>-187</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="12" t="n">
+        <v>756492</v>
+      </c>
+      <c r="D31" s="13" t="n">
+        <v>756492</v>
+      </c>
+      <c r="E31" s="19" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="H31" s="13" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>Rest of World excl. China</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="n">
+        <v>783495</v>
+      </c>
+      <c r="C32" s="12" t="n">
+        <v>381924</v>
+      </c>
+      <c r="D32" s="15" t="n">
+        <v>-401571</v>
+      </c>
+      <c r="E32" s="20" t="n">
+        <v>-0.513</v>
+      </c>
+      <c r="F32" s="12" t="n">
+        <v>313</v>
+      </c>
+      <c r="G32" s="12" t="n">
+        <v>114</v>
+      </c>
+      <c r="H32" s="15" t="n">
+        <v>-199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>